<commit_message>
feat(F-NAR-019): ATOM-DIF.ENE.001-03 Le château avant la soupe
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.ENE.001-03.xlsx
+++ b/stories/arbres/ATOM-DIF.ENE.001-03.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon puis cuisine, soupe de carotte</t>
+          <t>salon puis cuisine, soupe de carotte, vitre embuée, cuillère en bois, coussin rayé, casseroles tin tin</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut un château de coussins avant la soupe. Mila arrive avec beaucoup d'énergie. Le mur tombe. Elles jouent, elles attendent, Sarah demande à papa. Le château tient. La soupe est prête.</t>
+          <t>La cuillère en bois tape un bol. Au bord, un éclat de bol brille. Sarah veut un château de coussins, maintenant, avant la soupe. Mila saute trop, le mur tombe. Sourire parti, poitrine, papa accroupi. Sarah refuse de foncer, attend, demande. Merci vécu. Casseroles tin tin, cuillère trop vite. Un éclat de bol tient au bord.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un rond de vapeur s'ouvre sur la vitre. Dedans, le jardin est flou. Papa essuie un petit trou avec le doigt. Tu as senti la soupe, Sarah ? Oui. Ça sent la carotte. Maman plie une serviette chaude. On mange bientôt. Au salon, un coussin rayé a un carré de soleil. Le tissu est tiède. Une cuillère en bois attend près des bols. En ce moment, Sarah pose la joue sur le coussin. Je veux un château. Un château de coussins. On peut en faire un petit mur. Sarah pose un coussin. Puis un autre. Le mur est bas, un peu de travers. Mila arrive dans le salon. Elle court un peu. Elle saute. Elle a de l'énergie. Beaucoup d'énergie. Elle saute partout, papa. C'est son énergie. Ce n'est pas une faute. Mila pose un coussin trop vite. Le mur bascule. Un coussin glisse sur le tapis. Oh. Le château. Il peut se reconstruire. Sarah tient un coussin contre elle. Mila saute encore. Sarah regarde papa.</t>
+          <t>La cuillère en bois tape une fois contre un bol. Ça fait toc, sec et chaud. J'ai entendu le toc. Près des bols, Sarah ? Oui, papa. Un filet de vapeur monte vers la vitre. Papa essuie un petit trou avec le doigt. Le jardin est flou. Tu as senti la soupe, Sarah ? Ça sent la carotte. On mange bientôt. Maman plie une serviette chaude. Au bord du bol, un éclat de bol brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Au salon, un coussin rayé tient un carré de soleil. Le tissu est tiède, contre le visage. Il est chaud, papa. Le soleil est dessus ? Oui. En ce moment, Sarah pose un coussin. Je veux un château, maintenant ! Un château de coussins, avant la soupe. Un petit mur, là ? Oui, un mur. Les bols attendent, près de la vitre. Après le château. Sarah pose un autre coussin, plus haut. Le mur est bas, un peu de travers. Mila arrive dans le salon. Elle court un peu, pieds légers. Je saute ! Mila saute trop, trop près du mur. Tu poses avec moi ? Oui. Mila pose un coussin trop vite. Le mur bascule. Un coussin glisse sur le tapis. Oh. Le château. Il est tombé. Sarah tient un coussin contre elle. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Mila, Sarah ? Oui, papa. Tes mains tiennent le coussin, Sarah ? Un peu, maman. L'éclat de bol tremble, puis tient. Mila tape des pieds sur le tapis. Elle saute partout, papa. Sarah regarde papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un rond de vapeur s'ouvre sur la vitre. Dedans, le jardin est flou. Papa essuie un petit trou avec le doigt. Tu as senti la soupe, Sarah ? Oui. Ça sent la carotte. Maman plie une serviette chaude. On mange bientôt. Au salon, un coussin rayé a un carré de soleil. Le tissu est tiède. Une cuillère en bois attend près des bols. En ce moment, Sarah pose la joue sur le coussin. Je veux un château. Un château de coussins. On peut en faire un petit mur. Sarah pose un coussin. Puis un autre. Le mur est bas, un peu de travers. Mila arrive dans le salon. Elle court un peu. Elle saute. Elle a de l'énergie. Beaucoup d'énergie. Elle saute partout, papa. C'est son énergie. Ce n'est pas une faute. Mila pose un coussin trop vite. Le mur bascule. Un coussin glisse sur le tapis. Oh. Le château. Il peut se reconstruire. Sarah tient un coussin contre elle. Mila saute encore. Sarah regarde papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La cuillère en bois tape une fois contre un bol. Ça fait toc, sec et chaud. J'ai entendu le toc. Près des bols, Sarah ? Oui, papa. Un filet de vapeur monte vers la vitre. Papa essuie un petit trou avec le doigt. Le jardin est flou. Tu as senti la soupe, Sarah ? Ça sent la carotte. On mange bientôt. Maman plie une serviette chaude. Au bord du bol, un &lt;emphasis level="moderate"&gt;éclat de bol&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Au salon, un coussin rayé tient un carré de soleil. Le tissu est tiède, contre le visage. Il est chaud, papa. Le soleil est dessus ? Oui. En ce moment, Sarah pose un coussin. Je veux un château, maintenant ! Un château de coussins, avant la soupe. Un petit mur, là ? Oui, un mur. Les bols attendent, près de la vitre. Après le château. Sarah pose un autre coussin, plus haut. Le mur est bas, un peu de travers. Mila arrive dans le salon. Elle court un peu, pieds légers. Je saute ! Mila saute trop, trop près du mur. Tu poses avec moi ? Oui. Mila pose un coussin trop vite. Le mur bascule. Un coussin glisse sur le tapis. Oh. Le château. Il est tombé. Sarah tient un coussin contre elle. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Mila, Sarah ? Oui, papa. Tes mains tiennent le coussin, Sarah ? Un peu, maman. L'éclat de bol tremble, puis tient. Mila tape des pieds sur le tapis. Elle saute partout, papa. Sarah regarde papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sami est dans le salon. Papa est là. Maya arrive. Maya court un peu. Elle saute. Elle a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Beaucoup d'énergie. Ce n'est pas une faute. Sami la regarde. Papa dit : on peut jouer. On peut attendre. On peut demander à un adulte. Sami prend un coussin. Il dit : tu viens. Maya dit : oui. Ils font un petit mur. Maya pose vite. Sami attend son tour. Maya pose encore. L'énergie est là. Ce n'est pas une faute. Sami dit : on attend. Maya souffle. Elle attend. Puis papa sort des casseroles. Ils vont dans la cuisine. Maya tape un rythme. Sami se souvient. Il peut jouer. Il peut attendre. Il va vers papa. Il demande à un adulte. Papa dit : on se passe la cuillère en bois. Maya s'arrête. Elle tend les mains. Sami envoie la cuillère. Maya la renvoie. Ils jouent. Ils attendent, un peu. Papa dit : au salon, puis ici. C'est la même leçon. Maya a de l'énergie. Ce n'est pas une faute. On peut jouer. On peut attendre. Sami rit. Maya rit. [pause]</t>
+          <t>La cuillère en bois tape une fois contre un bol. Ça fait toc, sec et chaud. J'ai entendu le toc. Près des bols, Sarah ? Oui, papa. Un filet de vapeur monte vers la vitre. Papa essuie un petit trou avec le doigt. Le jardin est flou. Tu as senti la soupe, Sarah ? Ça sent la carotte. On mange bientôt. Maman plie une serviette chaude. Au bord du bol, un &lt;emphasis&gt;éclat de bol&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Au salon, un coussin rayé tient un carré de soleil. Le tissu est tiède, contre le visage. Il est chaud, papa. Le soleil est dessus ? Oui. En ce moment, Sarah pose un coussin. Je veux un château, maintenant ! Un château de coussins, avant la soupe. Un petit mur, là ? Oui, un mur. Les bols attendent, près de la vitre. Après le château. Sarah pose un autre coussin, plus haut. Le mur est bas, un peu de travers. Mila arrive dans le salon. Elle court un peu, pieds légers. Je saute ! Mila saute trop, trop près du mur. Tu poses avec moi ? Oui. Mila pose un coussin trop vite. Le mur bascule. Un coussin glisse sur le tapis. Oh. Le château. Il est tombé. Sarah tient un coussin contre elle. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Mila, Sarah ? Oui, papa. Tes mains tiennent le coussin, Sarah ? Un peu, maman. L'éclat de bol tremble, puis tient. Mila tape des pieds sur le tapis. Elle saute partout, papa. Sarah regarde papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>éclat de bol</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,44 +1321,73 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_un_chateau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un rond de vapeur s'ouvre sur la vitre.
-narrateur|Dedans, le jardin est flou.
+          <t>narrateur|La cuillère en bois tape une fois contre un bol.
+narrateur|Ça fait toc, sec et chaud.
+enfant-f|J'ai entendu le toc.
+papa|Près des bols, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Un filet de vapeur monte vers la vitre.
 narrateur|Papa essuie un petit trou avec le doigt.
+enfant-f|Le jardin est flou.
 papa|Tu as senti la soupe, Sarah ?
+enfant-f|Ça sent la carotte.
+maman|On mange bientôt.
+narrateur|Maman plie une serviette chaude.
+narrateur|Au bord du bol, un éclat de bol brille.
+enfant-f|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Au salon, un coussin rayé tient un carré de soleil.
+narrateur|Le tissu est tiède, contre le visage.
+enfant-f|Il est chaud, papa.
+papa|Le soleil est dessus ?
 enfant-f|Oui.
-enfant-f|Ça sent la carotte.
-narrateur|Maman plie une serviette chaude.
-maman|On mange bientôt.
-narrateur|Au salon, un coussin rayé a un carré de soleil.
-narrateur|Le tissu est tiède.
-narrateur|Une cuillère en bois attend près des bols.
-narrateur|En ce moment, Sarah pose la joue sur le coussin.
-enfant-f|Je veux un château.
-enfant-f|Un château de coussins.
-papa|On peut en faire un petit mur.
-narrateur|Sarah pose un coussin.
-narrateur|Puis un autre.
+narrateur|En ce moment, Sarah pose un coussin.
+enfant-f|Je veux un château, maintenant !
+enfant-f|Un château de coussins, avant la soupe.
+papa|Un petit mur, là ?
+enfant-f|Oui, un mur.
+maman|Les bols attendent, près de la vitre.
+enfant-f|Après le château.
+narrateur|Sarah pose un autre coussin, plus haut.
 narrateur|Le mur est bas, un peu de travers.
 narrateur|Mila arrive dans le salon.
-narrateur|Elle court un peu.
-narrateur|Elle saute.
-narrateur|Elle a de l'énergie.
-narrateur|Beaucoup d'énergie.
-enfant-f|Elle saute partout, papa.
-papa|C'est son énergie.
-papa|Ce n'est pas une faute.
+narrateur|Elle court un peu, pieds légers.
+copine|Je saute !
+narrateur|Mila saute trop, trop près du mur.
+enfant-f|Tu poses avec moi ?
+copine|Oui.
 narrateur|Mila pose un coussin trop vite.
 narrateur|Le mur bascule.
 narrateur|Un coussin glisse sur le tapis.
 enfant-f|Oh.
 enfant-f|Le château.
-maman|Il peut se reconstruire.
+copine|Il est tombé.
 narrateur|Sarah tient un coussin contre elle.
-narrateur|Mila saute encore.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Mila, Sarah ?
+enfant-f|Oui, papa.
+maman|Tes mains tiennent le coussin, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de bol tremble, puis tient.
+narrateur|Mila tape des pieds sur le tapis.
+enfant-f|Elle saute partout, papa.
 narrateur|Sarah regarde papa.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>coussin</t>
         </is>
       </c>
     </row>
@@ -1390,12 +1419,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Mila a de l'énergie. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila a de l'&lt;emphasis level="moderate"&gt;énergie&lt;/emphasis&gt;. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Maya a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que fait-on ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1458,18 +1487,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1484,11 +1513,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1499,23 +1528,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1524,23 +1553,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=mila_a_de_l_energie; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1573,17 +1602,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah va vers papa. Papa, on fait quoi ? On reconstruit le château. On joue, ou on attend un peu. Tu m'as demandé, je suis là. On se passe la cuillère en bois. Ils vont dans la cuisine. Les casseroles font tin tin. Mila tape un rythme sur ses genoux. Elle a encore de l'énergie. Ce n'est pas une faute. On peut attendre. Mila souffle. Elle tend les mains. Sarah envoie la cuillère. Mila la renvoie. La cuillère est lisse et chaude. Elles jouent. Puis elles reviennent au salon. Sarah pose un coussin. Elle attend. Mila pose le suivant. Le mur tient. Un coussin, puis l'autre. Le château. Il a une porte, là. Sarah glisse la main dans le trou. Le tissu est doux. La soupe chante tout bas. Un filet de vapeur monte. Tu as les mains sur la table, Sarah ? Oui, maman. Mila pose la cuillère. Elle attend.</t>
+          <t>Sarah veut le château, tout de suite. Je le refais, maintenant ! Elle avance trop vite vers Mila. Les mots se bousculent dans sa bouche. Attends. Mila tape des pieds, trop près. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le coussin, un instant. Elle écoute le toc de la cuillère. Tu veux le mur avec Mila ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose un coussin, puis l'autre. D'accord. Sarah pose le sien, sans se presser. Elle reste un moment, les mains ouvertes. Mila souffle. Le mien. Mila pose le suivant, plus lentement. Merci, Sarah. Papa a vu les deux, au salon. Le tissu est tiède, sous les doigts. Il est chaud. Le mur tient, un peu de travers. Le château. Il a une porte, là ? Oui, là. Sarah glisse la main dans le trou. Le tissu est doux, contre la peau. Tes mains sont au chaud, Sarah ? Un peu, maman. Mila s'assoit, puis se relève. J'y vais. On va à la cuisine ? La cuillère en bois est près des bols. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah va vers papa. Papa, on fait quoi ? On reconstruit le château. On joue, ou on attend un peu. Tu m'as demandé, je suis là. On se passe la cuillère en bois. Ils vont dans la cuisine. Les casseroles font tin tin. Mila tape un rythme sur ses genoux. Elle a encore de l'énergie. Ce n'est pas une faute. On peut attendre. Mila souffle. Elle tend les mains. Sarah envoie la cuillère. Mila la renvoie. La cuillère est lisse et chaude. Elles jouent. Puis elles reviennent au salon. Sarah pose un coussin. Elle attend. Mila pose le suivant. Le mur tient. Un coussin, puis l'autre. Le château. Il a une porte, là. Sarah glisse la main dans le trou. Le tissu est doux. La soupe chante tout bas. Un filet de vapeur monte. Tu as les mains sur la table, Sarah ? Oui, maman. Mila pose la cuillère. Elle attend.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah veut le &lt;emphasis level="moderate"&gt;château&lt;/emphasis&gt;, tout de suite. Je le refais, maintenant ! Elle avance trop vite vers Mila. Les mots se bousculent dans sa bouche. Attends. Mila tape des pieds, trop près. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le coussin, un instant. Elle écoute le toc de la cuillère. Tu veux le mur avec Mila ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose un coussin, puis l'autre. D'accord. Sarah pose le sien, sans se presser. Elle reste un moment, les mains ouvertes. Mila souffle. Le mien. Mila pose le suivant, plus lentement. Merci, Sarah. Papa a vu les deux, au salon. Le tissu est tiède, sous les doigts. Il est chaud. Le mur tient, un peu de travers. Le château. Il a une porte, là ? Oui, là. Sarah glisse la main dans le trou. Le tissu est doux, contre la peau. Tes mains sont au chaud, Sarah ? Un peu, maman. Mila s'assoit, puis se relève. J'y vais. On va à la cuisine ? La cuillère en bois est près des bols. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Maya a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Ce n'est pas une faute. Sami a joué. Il a su attendre. Il a demandé à papa. [pause]</t>
+          <t>Sarah veut le &lt;emphasis&gt;château&lt;/emphasis&gt;, tout de suite. Je le refais, maintenant ! Elle avance trop vite vers Mila. Les mots se bousculent dans sa bouche. Attends. Mila tape des pieds, trop près. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le coussin, un instant. Elle écoute le toc de la cuillère. Tu veux le mur avec Mila ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose un coussin, puis l'autre. D'accord. Sarah pose le sien, sans se presser. Elle reste un moment, les mains ouvertes. Mila souffle. Le mien. Mila pose le suivant, plus lentement. Merci, Sarah. Papa a vu les deux, au salon. Le tissu est tiède, sous les doigts. Il est chaud. Le mur tient, un peu de travers. Le château. Il a une porte, là ? Oui, là. Sarah glisse la main dans le trou. Le tissu est doux, contre la peau. Tes mains sont au chaud, Sarah ? Un peu, maman. Mila s'assoit, puis se relève. J'y vais. On va à la cuisine ? La cuillère en bois est près des bols. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1630,7 +1659,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1638,10 +1667,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1664,30 +1693,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>château</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1696,10 +1725,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1712,45 +1741,56 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_attend_demande; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah va vers papa.
+          <t>narrateur|Sarah veut le château, tout de suite.
+enfant-f|Je le refais, maintenant !
+narrateur|Elle avance trop vite vers Mila.
+narrateur|Les mots se bousculent dans sa bouche.
+copine|Attends.
+narrateur|Mila tape des pieds, trop près.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Sarah refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe le coussin, un instant.
+narrateur|Elle écoute le toc de la cuillère.
+papa|Tu veux le mur avec Mila ?
+narrateur|Papa reste à la même hauteur.
 enfant-f|Papa, on fait quoi ?
-papa|On reconstruit le château.
-papa|On joue, ou on attend un peu.
-papa|Tu m'as demandé, je suis là.
-maman|On se passe la cuillère en bois.
-narrateur|Ils vont dans la cuisine.
-narrateur|Les casseroles font tin tin.
-narrateur|Mila tape un rythme sur ses genoux.
-narrateur|Elle a encore de l'énergie.
-papa|Ce n'est pas une faute.
-enfant-f|On peut attendre.
+papa|On pose un coussin, puis l'autre.
+enfant-f|D'accord.
+narrateur|Sarah pose le sien, sans se presser.
+narrateur|Elle reste un moment, les mains ouvertes.
 narrateur|Mila souffle.
-narrateur|Elle tend les mains.
-narrateur|Sarah envoie la cuillère.
-narrateur|Mila la renvoie.
-narrateur|La cuillère est lisse et chaude.
-narrateur|Elles jouent.
-narrateur|Puis elles reviennent au salon.
-narrateur|Sarah pose un coussin.
-narrateur|Elle attend.
-narrateur|Mila pose le suivant.
-narrateur|Le mur tient.
-maman|Un coussin, puis l'autre.
+copine|Le mien.
+narrateur|Mila pose le suivant, plus lentement.
+papa|Merci, Sarah.
+narrateur|Papa a vu les deux, au salon.
+maman|Le tissu est tiède, sous les doigts.
+enfant-f|Il est chaud.
+narrateur|Le mur tient, un peu de travers.
 enfant-f|Le château.
-papa|Il a une porte, là.
+papa|Il a une porte, là ?
+enfant-f|Oui, là.
 narrateur|Sarah glisse la main dans le trou.
-narrateur|Le tissu est doux.
-narrateur|La soupe chante tout bas.
-narrateur|Un filet de vapeur monte.
-maman|Tu as les mains sur la table, Sarah ?
-enfant-f|Oui, maman.
-narrateur|Mila pose la cuillère.
-narrateur|Elle attend.</t>
+narrateur|Le tissu est doux, contre la peau.
+maman|Tes mains sont au chaud, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|Mila s'assoit, puis se relève.
+copine|J'y vais.
+enfant-f|On va à la cuisine ?
+maman|La cuillère en bois est près des bols.
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>coussin</t>
         </is>
       </c>
     </row>
@@ -1777,17 +1817,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On range ? Oui, papa. Sarah porte un coussin. Mila porte la cuillère. Vous posez ça près de la table ? Oui. Les bols attendent. La soupe est prête. Le château reste un peu, de travers. Il a tenu. Avant la soupe. Sarah souffle sur sa cuillère. La carotte sent bon.</t>
+          <t>Ils vont dans la cuisine. Les casseroles font tin tin. À moi ! Mila tape un rythme trop vite. On se passe la cuillère en bois ? Oui, maman. Sarah envoie la cuillère trop vite. La cuillère penche vers le bol. Ça tombe ! Attends. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le bol, un instant. Elle écoute le tin tin des casseroles. Au bord du bol, un éclat de bol luit. Là, sur le bol. Tu prends la cuillère, Mila ? Mila ne dit rien. Elle tend les mains, sans parler. Oui. Sarah envoie la cuillère, sans se presser. Mila la renvoie, plus lentement. La cuillère est lisse et chaude. Tu la vois, la cuillère ? Oui, papa. Les bols sont près de la vitre ? Oui, maman. Elles reviennent au salon. Sarah pose un coussin. Mila pose le suivant. Le mur tient, Sarah ? Oui, papa. Un rayon passe sur le tissu rayé. Il allume le château.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On range ? Oui, papa. Sarah porte un coussin. Mila porte la cuillère. Vous posez ça près de la table ? Oui. Les bols attendent. La soupe est prête. Le château reste un peu, de travers. Il a tenu. Avant la soupe. Sarah souffle sur sa cuillère. La carotte sent bon.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils vont dans la cuisine. Les casseroles font tin tin. À moi ! Mila tape un rythme trop vite. On se passe la cuillère en bois ? Oui, maman. Sarah envoie la cuillère trop vite. La cuillère penche vers le bol. Ça tombe ! Attends. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le bol, un instant. Elle écoute le tin tin des casseroles. Au bord du bol, un &lt;emphasis level="moderate"&gt;éclat de bol&lt;/emphasis&gt; luit. Là, sur le bol. Tu prends la cuillère, Mila ? Mila ne dit rien. Elle tend les mains, sans parler. Oui. Sarah envoie la cuillère, sans se presser. Mila la renvoie, plus lentement. La cuillère est lisse et chaude. Tu la vois, la cuillère ? Oui, papa. Les bols sont près de la vitre ? Oui, maman. Elles reviennent au salon. Sarah pose un coussin. Mila pose le suivant. Le mur tient, Sarah ? Oui, papa. Un rayon passe sur le tissu rayé. Il allume le château.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Papa dit : on range. Sami porte un coussin. Maya porte la cuillère. [pause]</t>
+          <t>Ils vont dans la cuisine. Les casseroles font tin tin. À moi ! Mila tape un rythme trop vite. On se passe la cuillère en bois ? Oui, maman. Sarah envoie la cuillère trop vite. La cuillère penche vers le bol. Ça tombe ! Attends. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le bol, un instant. Elle écoute le tin tin des casseroles. Au bord du bol, un &lt;emphasis&gt;éclat de bol&lt;/emphasis&gt; luit. Là, sur le bol. Tu prends la cuillère, Mila ? Mila ne dit rien. Elle tend les mains, sans parler. Oui. Sarah envoie la cuillère, sans se presser. Mila la renvoie, plus lentement. La cuillère est lisse et chaude. Tu la vois, la cuillère ? Oui, papa. Les bols sont près de la vitre ? Oui, maman. Elles reviennent au salon. Sarah pose un coussin. Mila pose le suivant. Le mur tient, Sarah ? Oui, papa. Un rayon passe sur le tissu rayé. Il allume le château. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1834,7 +1874,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1842,10 +1882,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1866,28 +1906,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de bol</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1896,10 +1940,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1910,22 +1954,55 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=casseroles_cuillere_trop_vite; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>papa|On range ?
+          <t>narrateur|Ils vont dans la cuisine.
+narrateur|Les casseroles font tin tin.
+copine|À moi !
+narrateur|Mila tape un rythme trop vite.
+maman|On se passe la cuillère en bois ?
+enfant-f|Oui, maman.
+narrateur|Sarah envoie la cuillère trop vite.
+narrateur|La cuillère penche vers le bol.
+enfant-f|Ça tombe !
+copine|Attends.
+narrateur|Sarah avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Sarah refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le bol, un instant.
+narrateur|Elle écoute le tin tin des casseroles.
+narrateur|Au bord du bol, un éclat de bol luit.
+enfant-f|Là, sur le bol.
+enfant-f|Tu prends la cuillère, Mila ?
+narrateur|Mila ne dit rien.
+narrateur|Elle tend les mains, sans parler.
+copine|Oui.
+narrateur|Sarah envoie la cuillère, sans se presser.
+narrateur|Mila la renvoie, plus lentement.
+narrateur|La cuillère est lisse et chaude.
+papa|Tu la vois, la cuillère ?
 enfant-f|Oui, papa.
-narrateur|Sarah porte un coussin.
-narrateur|Mila porte la cuillère.
-maman|Vous posez ça près de la table ?
-enfant-f|Oui.
-narrateur|Les bols attendent.
-papa|La soupe est prête.
-narrateur|Le château reste un peu, de travers.
-maman|Il a tenu.
-enfant-f|Avant la soupe.
-narrateur|Sarah souffle sur sa cuillère.
-narrateur|La carotte sent bon.</t>
+maman|Les bols sont près de la vitre ?
+enfant-f|Oui, maman.
+narrateur|Elles reviennent au salon.
+narrateur|Sarah pose un coussin.
+narrateur|Mila pose le suivant.
+papa|Le mur tient, Sarah ?
+enfant-f|Oui, papa.
+maman|Un rayon passe sur le tissu rayé.
+enfant-f|Il allume le château.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>casserole</t>
         </is>
       </c>
     </row>
@@ -1952,17 +2029,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Les bols sont chauds. Le château de coussins fait de l'ombre. Il attend après la soupe. On y retourne.</t>
+          <t>Ils restent près de la table. La soupe est prête, Sarah ? Oui, maman. Tu souffles sur ta cuillère ? Oui, papa. Sarah souffle, un filet de vapeur. La carotte sent bon. Tu la sens, la carotte ? Oui, maman. Le château reste un peu, de travers. Il a tenu, avant la soupe. Le château est resté. Les bols sont chauds, sous les mains. Le château de coussins fait de l'ombre. On y retourne, après. Un éclat de bol tient au bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Les bols sont chauds. Le château de coussins fait de l'ombre. Il attend après la soupe. On y retourne.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. La soupe est prête, Sarah ? Oui, maman. Tu souffles sur ta cuillère ? Oui, papa. Sarah souffle, un filet de vapeur. La carotte sent bon. Tu la sens, la carotte ? Oui, maman. Le château reste un peu, de travers. Il a tenu, avant la soupe. Le château est resté. Les bols sont chauds, sous les mains. Le château de coussins fait de l'ombre. On y retourne, après. Un &lt;emphasis level="moderate"&gt;éclat de bol&lt;/emphasis&gt; tient au bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. La soupe est prête, Sarah ? Oui, maman. Tu souffles sur ta cuillère ? Oui, papa. Sarah souffle, un filet de vapeur. La carotte sent bon. Tu la sens, la carotte ? Oui, maman. Le château reste un peu, de travers. Il a tenu, avant la soupe. Le château est resté. Les bols sont chauds, sous les mains. Le château de coussins fait de l'ombre. On y retourne, après. Un &lt;emphasis&gt;éclat de bol&lt;/emphasis&gt; tient au bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2009,18 +2086,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2029,12 +2106,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2043,17 +2120,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de bol</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2062,11 +2143,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2075,27 +2156,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_au_bord; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Les bols sont chauds.
+          <t>narrateur|Ils restent près de la table.
+maman|La soupe est prête, Sarah ?
+enfant-f|Oui, maman.
+papa|Tu souffles sur ta cuillère ?
+enfant-f|Oui, papa.
+narrateur|Sarah souffle, un filet de vapeur.
+enfant-f|La carotte sent bon.
+maman|Tu la sens, la carotte ?
+enfant-f|Oui, maman.
+papa|Le château reste un peu, de travers.
+enfant-f|Il a tenu, avant la soupe.
+copine|Le château est resté.
+narrateur|Les bols sont chauds, sous les mains.
 narrateur|Le château de coussins fait de l'ombre.
-papa|Il attend après la soupe.
-enfant-f|On y retourne.</t>
+enfant-f|On y retourne, après.
+narrateur|Un éclat de bol tient au bord.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>soupe</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2201,6 +2303,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>